<commit_message>
Publish 2026-09-18 04:47 UTC (src 6ee7bda)
</commit_message>
<xml_diff>
--- a/Data/Capital_Budgeting_Solution.xlsx
+++ b/Data/Capital_Budgeting_Solution.xlsx
@@ -1,66 +1,58 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Model" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Model" sheetId="1" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_adj" vbProcedure="false">Model!$B$10:$F$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_cvg" vbProcedure="false">0.0001</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_drv" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_eng" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_est" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_itr" vbProcedure="false">2147483647</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lhs1" vbProcedure="false">Model!$H$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lhs2" vbProcedure="false">Model!$H$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lhs3" vbProcedure="false">Model!$H$6</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lhs4" vbProcedure="false">Model!$H$7</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lhs5" vbProcedure="false">Model!$B$10:$F$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_lin" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_mip" vbProcedure="false">2147483647</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_mni" vbProcedure="false">30</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_mrt" vbProcedure="false">0.075</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_msl" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_ncr" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_neg" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_nod" vbProcedure="false">2147483647</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_num" vbProcedure="false">5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_nwt" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_opt" vbProcedure="false">Model!$H$13</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_pre" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rel1" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rel2" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rel3" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rel4" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rel5" vbProcedure="false">5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rhs1" vbProcedure="false">Model!$J$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rhs2" vbProcedure="false">Model!$J$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rhs3" vbProcedure="false">Model!$J$6</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rhs4" vbProcedure="false">Model!$J$7</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rhs5" vbProcedure="false">binary</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rlx" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_rsd" vbProcedure="false">0</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_scl" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_show" vbProcedure="false">2</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_sol" vbProcedure="false">2147483647</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_ssz" vbProcedure="false">100</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_tim" vbProcedure="false">2147483647</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_tol" vbProcedure="false">0</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_typ" vbProcedure="false">1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="solver_ver" vbProcedure="false">3</definedName>
+    <definedName name="solver_adj" hidden="true" localSheetId="0">Model!$B$10:$F$10</definedName>
+    <definedName name="solver_cvg" hidden="true" localSheetId="0">0.0001</definedName>
+    <definedName name="solver_drv" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_eng" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_est" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_itr" hidden="true" localSheetId="0">2147483647</definedName>
+    <definedName name="solver_lhs1" hidden="true" localSheetId="0">Model!$H$4</definedName>
+    <definedName name="solver_lhs2" hidden="true" localSheetId="0">Model!$H$5</definedName>
+    <definedName name="solver_lhs3" hidden="true" localSheetId="0">Model!$H$6</definedName>
+    <definedName name="solver_lhs4" hidden="true" localSheetId="0">Model!$H$7</definedName>
+    <definedName name="solver_lhs5" hidden="true" localSheetId="0">Model!$B$10:$F$10</definedName>
+    <definedName name="solver_lin" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_mip" hidden="true" localSheetId="0">2147483647</definedName>
+    <definedName name="solver_mni" hidden="true" localSheetId="0">30</definedName>
+    <definedName name="solver_mrt" hidden="true" localSheetId="0">0.075</definedName>
+    <definedName name="solver_msl" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_ncr" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_neg" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_nod" hidden="true" localSheetId="0">2147483647</definedName>
+    <definedName name="solver_num" hidden="true" localSheetId="0">5</definedName>
+    <definedName name="solver_nwt" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_opt" hidden="true" localSheetId="0">Model!$H$13</definedName>
+    <definedName name="solver_pre" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_rel1" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_rel2" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_rel3" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_rel4" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_rel5" hidden="true" localSheetId="0">5</definedName>
+    <definedName name="solver_rhs1" hidden="true" localSheetId="0">Model!$J$4</definedName>
+    <definedName name="solver_rhs2" hidden="true" localSheetId="0">Model!$J$5</definedName>
+    <definedName name="solver_rhs3" hidden="true" localSheetId="0">Model!$J$6</definedName>
+    <definedName name="solver_rhs4" hidden="true" localSheetId="0">Model!$J$7</definedName>
+    <definedName name="solver_rhs5" hidden="true" localSheetId="0">binary</definedName>
+    <definedName name="solver_rlx" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_rsd" hidden="true" localSheetId="0">0</definedName>
+    <definedName name="solver_scl" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_show" hidden="true" localSheetId="0">2</definedName>
+    <definedName name="solver_sol" hidden="true" localSheetId="0">2147483647</definedName>
+    <definedName name="solver_ssz" hidden="true" localSheetId="0">100</definedName>
+    <definedName name="solver_tim" hidden="true" localSheetId="0">2147483647</definedName>
+    <definedName name="solver_tol" hidden="true" localSheetId="0">0</definedName>
+    <definedName name="solver_typ" hidden="true" localSheetId="0">1</definedName>
+    <definedName name="solver_ver" hidden="true" localSheetId="0">3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -591,23 +583,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="14"/>
+    <col min="1" max="1" width="30" customWidth="true"/>
+    <col min="2" max="10" width="14" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>1</v>
@@ -633,7 +622,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -664,7 +653,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -695,7 +684,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6">
       <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
@@ -726,7 +715,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -757,7 +746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
@@ -777,7 +766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
@@ -797,7 +786,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13">
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
@@ -824,43 +813,37 @@
         <v>330</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15">
       <c r="A15" s="14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16">
       <c r="A16" s="14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17">
       <c r="A17" s="14" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18">
       <c r="A18" s="14" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19">
       <c r="A19" s="14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20">
       <c r="A20" s="14" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>